<commit_message>
Record the E15-S12 re-promotion and SIT re-run on the story
QA CI on 4426069 was red on the dependency audit, not on the story's code;
fixed in 2125817. Re-promoted to QA e28427e, CI green on DEV and QA.
SIT re-run against the QA tree: 201 passed, 0 failed (181 SIT including
the 7 SIT-20 scenarios, plus the 20 dependency-hygiene tests), algotrader
loaded from the QA worktree. No new SIT defects.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documents/BACKLOG_Tracker.xlsx
+++ b/Documents/BACKLOG_Tracker.xlsx
@@ -21336,7 +21336,9 @@
 QA-E15-23 (CRITICAL, in E15-S09's shipped code) FIXED HERE: only a WORKING exit covers a holding. Anything uncovered once the day's exit key is spent (EXIT_SPENT), or our exits outrunning our entries (OVER_EXITED), halts once and re-arms every cycle.
 FOUND DURING THE STORY: two E15-S09 tests asserted what the fake allowed and the real key rule forbids (QA-E15-24); PositionManager accepted no calendar and failed at its first booking (QA-E15-25); an integration helper committed its session and leaked rows into the next file (QA-E15-26); a mutation survivor's test passed for the wrong reason (QA-E15-27); a booking failure's broker text reached the audit table (REC-003).
 TESTS: 2,361 -&gt; 2,419; coverage 93% flat; 30 reconciler unit + 8 position-manager unit + 9 gateway-cancel unit + 4 integration (real Postgres, Redis, Kite mapping) + 7 SIT-20. Mutation: 21 injected, 21 killed (19/21 first run; both survivors verified benign - second layers - and now held directly).
-SIT AGAINST THE PROMOTED QA TREE, 15 Oct 2026: QA 4426069 (DEV 21c042c, CI green on DEV). 181 passed, 0 failed, including all 7 SIT-20 scenarios; Documents/, scripts/tracker and .claude absent from the QA tree.</t>
+SIT AGAINST THE PROMOTED QA TREE, 15 Oct 2026: QA 4426069 (DEV 21c042c, CI green on DEV). 181 passed, 0 failed, including all 7 SIT-20 scenarios; Documents/, scripts/tracker and .claude absent from the QA tree.
+QA CI ON 4426069 WAS RED, 15 Oct 2026 - not this story's code. The Tests job passed; the Security job's dependency audit failed on four advisories published between the DEV run (30 Sep) and the QA run: three in urllib3 2.7.0 and one in Twisted 26.4.0 (DEP-001, DEP-002, DEP-003). Fixed in DEV 2125817 - urllib3 2.8.0; the Twisted IMAP-server advisory, which has no patched release and is unreachable here, is ignored by ID and the ignore is held by TestTheAcceptedTwistedAdvisory. Full gate 2,427 passed, 0 skipped, coverage 93%.
+RE-PROMOTED AND SIT RE-RUN, 15 Oct 2026: QA e28427e (DEV 2125817), CI green on DEV and QA. 201 passed, 0 failed - all 181 SIT scenarios including the 7 SIT-20 ones, plus the 20 dependency-hygiene tests - run from a worktree of the QA branch with algotrader confirmed loaded from that tree. Documents/, scripts/tracker and .claude absent from QA. No new SIT defects.</t>
         </is>
       </c>
       <c r="W204" s="49" t="n"/>

</xml_diff>

<commit_message>
Record E15-S13's QA run; the skill now runs gitleaks before a push
E15-S13 is QA-Success: DEV 83cd00b (CI Run 115) promoted to QA 12c42cf
(CI Run 116); the whole suite on the QA tree passed, 2,731 with none
skipped, SIT-21 included. Tracker: QA-E15-29..33, AUDIT-026..029, the
new E15-S14 (live ATR and per-share margin), and this story's
constraints written onto E15-S10, E23-S03, E13-S04, E20-S05, E04-S05.

Skill Phase 7: CI Run 114 failed on a gitleaks finding no local gate
could see. The skill now scans the unpushed range with the gitleaks
container and records the fixture convention.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documents/BACKLOG_Tracker.xlsx
+++ b/Documents/BACKLOG_Tracker.xlsx
@@ -21393,7 +21393,7 @@
       </c>
       <c r="E205" s="40" t="inlineStr">
         <is>
-          <t>Development Completed</t>
+          <t>QA-Success</t>
         </is>
       </c>
       <c r="F205" s="41" t="inlineStr">
@@ -21464,9 +21464,9 @@
 AC REWRITTEN AS FALSIFIABLE: AC1 = a Recommendation published on stream:signals, consumed by the running service against the real adapter/Postgres/Redis, is submitted, and after the broker fills it the next cycle holds a ProtectedPosition under the signal's correlation with an SL-M stop for the filled quantity. AC2 = with the kill switch armed in Redis (or any rejection), no order row exists and the broker received nothing. AC3 = start() restores before the first cycle; a held position is in the book after the first cycle and no exit is sent; signals are refused until a cycle has succeeded.
 DELIVERED 28 Oct 2026: execution/service.py (ExecutionService, RedisSignalSource), execution/session_context.py (RiskContextBuilder, PendingEntries, PendingAwareSlots, NoProducerYet, RepositoryContextStore), execution/risk/factory.py (build_risk_engine - the only RiskEngine constructor in src, asserted by AST), ReconciliationLoop(guard=...), reconciliation forgets an ENTRY's plan when it writes SUBMIT_FAILED, InstrumentRepository.profile, PositionRepository.closed_since, ExecutionConfig.max_signal_age_seconds (hard cap MAX_SIGNAL_AGE_SECONDS=300).
 DECISIONS: one asyncio lock for signals and cycles (9.1 made structural); sent-not-booked entries count as held, slotted and exposed; plans registered BEFORE the broker call; unknown send outcomes keep the plan, definitive ones release it; duplicates (row exists or ledger unreadable) are refused, never re-evaluated; VETO, stale (&gt;60s default) and future-dated (&gt;5s) signals, alert_only and approval modes are refused before the engine and audited under stage EXECUTION; all four surveillance flags block (recorded assumption); a missing daily row assumes the earlier CAS deadline and leaves eligibility unknown.
-GATES: Full gate 28 Oct 2026: 2,731 passed, 0 failed, 0 skipped, coverage 93% (flat; service 95%, session_context 93%, factory 100%, reconciliation 96%); ruff check/format and mypy clean over the whole tree; bandit 0; pip-audit clean (7 accepted IDs); security suite 460 passed; doctor: Configuration/Broker SDK/Market calendar/Strategies OK (Datastores FAIL and Secrets/SEBI/Network WARN are the dev machine).
+GATES: Full gate 28 Oct 2026: 2,731 passed, 0 failed, 0 skipped, coverage 93% (flat; service 95%, session_context 93%, factory 100%, reconciliation 96%); ruff check/format and mypy clean over the whole tree; bandit 0; pip-audit clean (7 accepted IDs), re-run before push; security suite 460 passed; gitleaks clean on the pushed range; doctor: Configuration/Broker SDK/Market calendar/Strategies OK (Datastores FAIL and Secrets/SEBI/Network WARN are the dev machine). CI: DEV Run 114 FAILED (gitleaks, QA-E15-33) -&gt; fixed in 83cd00b -&gt; DEV Run 115 green; promoted DEV 83cd00b -&gt; QA 12c42cf via promote.py (CI check passed, no divergence, Documents/scripts/tracker/.claude stripped and verified absent); QA Run 116 green.
 MUTATION: 34 named mutations, 34 killed after QA-E15-32 (one test passing for the wrong reason fixed; one redundant release removed; one anchor corrected); sources byte-identical.
-SIT: Pending - SIT-21 (tests/sit/test_e15_execution_session.py: a whole day, a restart mid-session, a kill switch mid-session) passed on DEV; to run on the QA tree.</t>
+SIT: SIT on the QA tree (worktree at origin/QA 12c42cf, algotrader imported from the worktree), whole suite because the change spans components: 2,731 passed, 0 failed, 0 skipped. SIT-21 (tests/sit/test_e15_execution_session.py) walks a whole day through the real stack - pre-open, both no-trade windows, a duplicate delivery, a missing daily row, a VETO, a stale signal, a held symbol - and asserts every signal ends exactly one audited way, every entry is protected by one stop, nothing is exited, no halt; plus a restart mid-session (book kept, nothing placed, next signal gets slot 2) and a kill switch mid-session (new entries refused, protection untouched). No SIT defects.</t>
         </is>
       </c>
       <c r="W205" s="49" t="n"/>
@@ -22339,7 +22339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J154"/>
+  <dimension ref="A1:J155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="59" min="1" max="1"/>
@@ -22367,6 +22367,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="82" t="inlineStr">
         <is>
@@ -28059,6 +28060,43 @@
       <c r="G154" s="76" t="inlineStr">
         <is>
           <t>34/34 killed; sources byte-identical after every run. tests/unit/test_session_context.py::TestPendingEntries::test_every_read_prunes_first[len|contains|entries|slots].</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="76" t="inlineStr">
+        <is>
+          <t>QA-E15-33</t>
+        </is>
+      </c>
+      <c r="B155" s="76" t="inlineStr">
+        <is>
+          <t>E15-S13</t>
+        </is>
+      </c>
+      <c r="C155" s="76" t="inlineStr">
+        <is>
+          <t>CI's secret scan failed a commit every local gate had passed</t>
+        </is>
+      </c>
+      <c r="D155" s="76" t="inlineStr">
+        <is>
+          <t>FAIL -&gt; Fixed</t>
+        </is>
+      </c>
+      <c r="E155" s="76" t="inlineStr">
+        <is>
+          <t>DEV CI Run 114 (b14532c) failed its Security job: gitleaks generic-api-key, twice, on a test fixture written as one literal ('api_key=... access_token=...') in TestNothingSecretReachesTheAuditTable. Fake values, nothing to rotate. The local Phase 7 gate runs bandit, pip-audit and the security suite - not gitleaks - so it could not see it: AUDIT-022's 'the local gate is not CI's gate', one job over.</t>
+        </is>
+      </c>
+      <c r="F155" s="76" t="inlineStr">
+        <is>
+          <t>Reproduced locally with the gitleaks container (2 findings, same rule and line). Fixtures assembled at runtime with a comment, the convention test_log_redaction.py already uses (83cd00b); the unpushed range then scanned clean, and CI Run 115 passed - which also confirmed the action judges each push on its own, so b14532c stays in history without a force-push. The /sdlc skill's Phase 7 now runs gitleaks on the unpushed range.</t>
+        </is>
+      </c>
+      <c r="G155" s="76" t="inlineStr">
+        <is>
+          <t>CI Run 115 (DEV 83cd00b) green; local gitleaks over every file this story added: no leaks found.</t>
         </is>
       </c>
     </row>
@@ -28108,6 +28146,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Reconcile the tracker against the code
Six stories were New with work in the code: E04-S07 (the 2026 holiday
list, verified), E21-S08 (verify_chain), E22-S02 (the Testcontainers
integration suite), E23-S05 (CI), E20-S01 (13 metrics) and E21-S02 (the
static-IP and egress checks). Each is now Development Completed with
its evidence and its remainder on the row. Seven more carry an evidence
note with the status unchanged, including a scope correction on E22-S07
(it names execution/risk_engine.py, which does not exist). The header
now counts 202 stories.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documents/BACKLOG_Tracker.xlsx
+++ b/Documents/BACKLOG_Tracker.xlsx
@@ -4568,7 +4568,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: BACKLOG.md · 189 stories across 24 epics · Set Status from the dropdown in column E. Yellow-tinted columns (M–Q, W) are yours to fill in. Tasks/Acceptance are wrapped — widen a row or click a cell to read the full text.</t>
+          <t>Source: BACKLOG.md · 202 stories across 24 epics (189 from BACKLOG.md, 13 raised since) · Set Status from the dropdown in column E. Yellow-tinted columns (M–Q, W) are yours to fill in. Tasks/Acceptance are wrapped — widen a row or click a cell to read the full text.</t>
         </is>
       </c>
     </row>
@@ -7614,7 +7614,11 @@
       </c>
       <c r="T37" s="48" t="n"/>
       <c r="U37" s="48" t="n"/>
-      <c r="V37" s="48" t="n"/>
+      <c r="V37" s="48" t="inlineStr">
+        <is>
+          <t>TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Status unchanged (New). common/db/retention.py archives BARS (ohlcv) to Parquet (E01-S06); nothing archives ticks.</t>
+        </is>
+      </c>
       <c r="W37" s="49" t="n"/>
     </row>
     <row r="38" ht="30" customHeight="1" s="59">
@@ -8143,7 +8147,7 @@
       </c>
       <c r="E44" s="40" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Development Completed</t>
         </is>
       </c>
       <c r="F44" s="41" t="inlineStr">
@@ -8205,7 +8209,8 @@
       </c>
       <c r="V44" s="48" t="inlineStr">
         <is>
-          <t>DATED, 27 Oct 2026: config/nse_holidays.yaml covers 2026 only. MarketCalendar fails CLOSED on an uncovered year (HolidayDataError), so from 1 Jan 2027 the system refuses to trade until the 2027 list is added. NSE publishes it in December; add it, triangulated against two publications as the 2026 list was, before the last trading day of 2026.</t>
+          <t>DATED, 27 Oct 2026: config/nse_holidays.yaml covers 2026 only. MarketCalendar fails CLOSED on an uncovered year (HolidayDataError), so from 1 Jan 2027 the system refuses to trade until the 2027 list is added. NSE publishes it in December; add it, triangulated against two publications as the 2026 list was, before the last trading day of 2026.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Was New; the work was done on 24 Aug 2026 and never recorded. config/nse_holidays.yaml transcribes NSE's 2026 list (21 dates), verified_against_nse_circular: true, covers_years: [2026]; the Muhurat Sunday session is modelled in common/calendar.py; doctor.py reports the list verified. DELIVERED IN PART - remaining: (1) the 2027 list before the last trading day of 2026 (the calendar fails closed on an uncovered year, see the dated note above); (2) the runbook reminder (E23-S06, unbuilt); (3) automated fetch was 'consider' and is not built.</t>
         </is>
       </c>
       <c r="W44" s="49" t="n"/>
@@ -9117,7 +9122,8 @@
       <c r="V54" s="48" t="inlineStr">
         <is>
           <t>EMA, SMA, RSI, MACD, ATR, Bollinger, VWAP, VolumeRatio - all matched to TA-Lib within 1e-4. MACD needed a real fix found by that comparison: TA-Lib seeds BOTH its EMAs at the same bar (the slow period's start), not each at its own. Composing two independent EMAs read -18.75 where TA-Lib read -20.11 on a 200-bar series - a 7% error on a line whose CROSSINGS are the signal. Bollinger uses population not sample stddev (2.6% apart at n=20). VWAP is session-anchored and ignores synthetic bars. VolumeRatio excludes the current bar so a 10x spike does not damp itself.
-NOT DONE: ADX. Listed in the story, deferred - it is the only one with no consumer yet.</t>
+NOT DONE: ADX. Listed in the story, deferred - it is the only one with no consumer yet.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Status confirmed (Development Completed): still no ADX in indicators/ (engine.py, framework.py, levels.py).</t>
         </is>
       </c>
       <c r="W54" s="49" t="n"/>
@@ -12832,7 +12838,11 @@
         </is>
       </c>
       <c r="U100" s="48" t="n"/>
-      <c r="V100" s="48" t="n"/>
+      <c r="V100" s="48" t="inlineStr">
+        <is>
+          <t>TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Status unchanged (New). The strategy and strategy_trial tables exist (E01 schema) and strategy documents compile from config/strategies (scripts/validate_strategies.py), but there is no repository, no persistence of a StrategyDocument and no load-on-startup.</t>
+        </is>
+      </c>
       <c r="W100" s="49" t="n"/>
     </row>
     <row r="101" ht="30" customHeight="1" s="59">
@@ -18436,7 +18446,7 @@
       </c>
       <c r="E167" s="40" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Development Completed</t>
         </is>
       </c>
       <c r="F167" s="53" t="inlineStr">
@@ -18477,7 +18487,8 @@
       <c r="U167" s="48" t="n"/>
       <c r="V167" s="48" t="inlineStr">
         <is>
-          <t>Latency histograms per stage · data quality counters · AI metrics including cache hit ratio · trading counters · risk gauges · health.</t>
+          <t>Latency histograms per stage · data quality counters · AI metrics including cache hit ratio · trading counters · risk gauges · health.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Was New. common/metrics.py registers 13 Prometheus metrics: signals_approved/rejected_total, risk_check_errors_total, risk_evaluation_seconds, positions_opened_total, partial_fills_total, naked_positions_total, unprotectable_fills_total, stop_attach_failures_total, unknown_positions_total, reconciliation_cycles/drift/read_failures_total. DELIVERED IN PART - remaining: per-stage latency histograms (only the risk evaluation has one), data-quality counters, AI metrics incl. cache hit ratio, health.</t>
         </is>
       </c>
       <c r="W167" s="49" t="n"/>
@@ -18852,7 +18863,8 @@
       <c r="U172" s="48" t="n"/>
       <c r="V172" s="48" t="inlineStr">
         <is>
-          <t>Correlation ID binding across all services.</t>
+          <t>Correlation ID binding across all services.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Status unchanged (New). common/logging.py provides bind_correlation() (E00-S05), but nothing in src calls it: no service binds a correlation id yet.</t>
         </is>
       </c>
       <c r="W172" s="49" t="n"/>
@@ -18957,7 +18969,7 @@
       </c>
       <c r="E174" s="40" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Development Completed</t>
         </is>
       </c>
       <c r="F174" s="41" t="inlineStr">
@@ -18998,7 +19010,8 @@
       <c r="U174" s="48" t="n"/>
       <c r="V174" s="48" t="inlineStr">
         <is>
-          <t>Compare actual egress IP against config; refuse to start on mismatch in live mode.</t>
+          <t>Compare actual egress IP against config; refuse to start on mismatch in live mode.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Was New. AppConfig refuses to load in LIVE mode without system.static_ip; scripts/doctor.py:check_egress_ip compares the actual egress IP with EXPECTED_EGRESS_IP (warns when unset). DELIVERED IN PART - remaining: 'refuse to START on mismatch' belongs to a service entrypoint, and none exists yet (E23-S03).</t>
         </is>
       </c>
       <c r="W174" s="49" t="n"/>
@@ -19411,7 +19424,7 @@
       </c>
       <c r="E180" s="40" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Development Completed</t>
         </is>
       </c>
       <c r="F180" s="53" t="inlineStr">
@@ -19456,7 +19469,8 @@
       <c r="U180" s="48" t="n"/>
       <c r="V180" s="48" t="inlineStr">
         <is>
-          <t>Verify the hash chain end to end; detect any retroactive modification.</t>
+          <t>Verify the hash chain end to end; detect any retroactive modification.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Was New. common/audit.py:verify_chain verifies the hash chain end to end and detects retroactive modification (built under E01-S05; tests/integration/test_audit_chain.py incl. hypothesis tampering cases). DELIVERED IN PART - remaining: the operator-facing utility (a command or script that runs it and reports) and a schedule; neither exists.</t>
         </is>
       </c>
       <c r="W180" s="49" t="n"/>
@@ -19535,7 +19549,11 @@
         </is>
       </c>
       <c r="U181" s="48" t="n"/>
-      <c r="V181" s="48" t="n"/>
+      <c r="V181" s="48" t="inlineStr">
+        <is>
+          <t>TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Status unchanged (New). Task 1 exists, built under E14-S07: tests/unit/test_sizer.py's hypothesis property that sizing never rounds up (risk never exceeds budget). Tasks 2-5 (slot count, approved-has-stop, square-off before the broker's deadline, monotonic clamps) have no property tests.</t>
+        </is>
+      </c>
       <c r="W181" s="49" t="n"/>
     </row>
     <row r="182" ht="30" customHeight="1" s="59">
@@ -19561,7 +19579,7 @@
       </c>
       <c r="E182" s="40" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Development Completed</t>
         </is>
       </c>
       <c r="F182" s="53" t="inlineStr">
@@ -19602,7 +19620,8 @@
       <c r="U182" s="48" t="n"/>
       <c r="V182" s="48" t="inlineStr">
         <is>
-          <t>Testcontainers for Redis and Postgres; every inter-service contract exercised.</t>
+          <t>Testcontainers for Redis and Postgres; every inter-service contract exercised.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Was New. The Testcontainers harness for Postgres and Redis exists (tests/conftest.py) with 21 integration files (~9,800 lines) - persistence, audit chain, broker rate limit, gateway, order state, protective stop, positions, reconciliation, slots, tick-to-trigger, the execution service - and CI runs them on every push. DELIVERED IN PART - remaining: the contracts of services not built yet (signal engine, AI, pre-market, macro, notifier, API).</t>
         </is>
       </c>
       <c r="W182" s="49" t="n"/>
@@ -19675,7 +19694,8 @@
       <c r="U183" s="48" t="n"/>
       <c r="V183" s="48" t="inlineStr">
         <is>
-          <t>Replay a recorded session through the full pipeline; assert deterministic outputs; regression on every change.</t>
+          <t>Replay a recorded session through the full pipeline; assert deterministic outputs; regression on every change.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Status unchanged (New). tests/replay contains only __init__.py.</t>
         </is>
       </c>
       <c r="W183" s="49" t="n"/>
@@ -19753,7 +19773,8 @@
       </c>
       <c r="V184" s="48" t="inlineStr">
         <is>
-          <t>All nine scenarios from LOW_LEVEL_ARCHITECTURE §12.3 — kill each service, Redis restart, WebSocket drop, AI outage, broker 500, clock jump, disk full, duplicate tick flood.</t>
+          <t>All nine scenarios from LOW_LEVEL_ARCHITECTURE §12.3 — kill each service, Redis restart, WebSocket drop, AI outage, broker 500, clock jump, disk full, duplicate tick flood.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Status unchanged (New). tests/chaos contains only __init__.py; degraded-dependency scenarios live in tests/sit instead.</t>
         </is>
       </c>
       <c r="W184" s="49" t="n"/>
@@ -19964,7 +19985,8 @@
       <c r="U187" s="48" t="n"/>
       <c r="V187" s="48" t="inlineStr">
         <is>
-          <t>100% line coverage gate on `execution/risk_engine.py` and `execution/sizer.py`.</t>
+          <t>100% line coverage gate on `execution/risk_engine.py` and `execution/sizer.py`.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Status unchanged (New) - no coverage gate exists anywhere (no fail_under in pyproject, Makefile or ci.yml). Today the modules this story means are covered: execution/risk/checks/* 100%, factory 100%, framework 99%, sizer 100% (full gate, 28 Oct 2026) - nothing keeps them there. CORRECTION to the scope: the story names execution/risk_engine.py, which does not exist - the engine is execution/risk/ (framework.py, checks/, factory.py). pyproject's [tool.coverage.paths] 'risk' entry names the same missing file and is not an enforcement mechanism ([paths] maps source locations when combining data files).</t>
         </is>
       </c>
       <c r="W187" s="49" t="n"/>
@@ -20359,7 +20381,7 @@
       </c>
       <c r="E193" s="40" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Development Completed</t>
         </is>
       </c>
       <c r="F193" s="53" t="inlineStr">
@@ -20400,7 +20422,8 @@
       <c r="U193" s="48" t="n"/>
       <c r="V193" s="48" t="inlineStr">
         <is>
-          <t>`make check` on every PR; gitleaks; pip-audit; safety-invariant tests as a required check on `QA` and `PROD`.</t>
+          <t>`make check` on every PR; gitleaks; pip-audit; safety-invariant tests as a required check on `QA` and `PROD`.
+TRACKER RECONCILED AGAINST THE CODE, 28 Oct 2026: Was New. .github/workflows/ci.yml runs on push and pull_request to DEV/QA/PROD/main: lint/format/types (make check's commands), tests incl. tests/security (the safety invariants), gitleaks, pip-audit with assessed ignores, a container image build, and a CI-gate job; scripts/promote.py refuses a DEV-&gt;QA promotion unless CI passed on the commit. DELIVERED IN PART - remaining: 'a required check on QA and PROD' needs GitHub branch protection, which is off on every branch (checked 28 Oct 2026) - the owner's action, and recommended.</t>
         </is>
       </c>
       <c r="W193" s="49" t="n"/>
@@ -22367,7 +22390,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="82" t="inlineStr">
         <is>
@@ -28146,7 +28168,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Record E15-S06's QA run
E15-S06 is QA-Success: DEV 4c1ab92 (CI Run 119) promoted to QA a9c971b
(CI Run 120); the whole suite on the QA tree passed, 2,798 with none
skipped and pytest exit 0, SIT-21 and SIT-22 included. No SIT defects.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documents/BACKLOG_Tracker.xlsx
+++ b/Documents/BACKLOG_Tracker.xlsx
@@ -15710,7 +15710,7 @@
       </c>
       <c r="E132" s="40" t="inlineStr">
         <is>
-          <t>Development Completed</t>
+          <t>QA-Success</t>
         </is>
       </c>
       <c r="F132" s="41" t="inlineStr">
@@ -15779,9 +15779,9 @@
 OUT OF SCOPE, recorded: exit precedence beyond 'a triggered stop is the exit' (E15-S07); reducing quantity on partial exits (E15-S08 - a stop that part-fills then cancels is exited for the remainder and HALTS as not held); alert transports (E19); the process entrypoint (E23-S03).
 DECISIONS: (1) Task 2's Redis sorted set NOT built - a second copy of the deadline, and a missed add is a position with no time exit; the sweep reads the book. LLA 5.8 rewritten. (2) Constraint 4: the timer SHARES the SQUAREOFF key - unused for every position it acts on, no migration of order_intent_enum, no second exit key. (3) Constraint 5: cancel the stop and send nothing until the broker shows it terminal (CANCEL PENDING maps to OPEN = live, so the reconciler cannot add an exit in the gap either). (4) Constraints 2-3: ExitingPosition gains reason; reconciliation closes with it (TIME / UNPROTECTED). (5) Build concern 1: one-second loop + backstop sweep after every cycle and reconnect + stall detection (squareoff_timer_stalls_total). (6) Build concern 2: the exit is MARKET with market_protection (asserted at the Kite payload). (7) Every exit min(book, broker): see AUDIT-030. (8) A halt never stops the timer.
 RESIDUALS, recorded: after a restart mid time-exit the close may read UNPROTECTED (the reason is in memory); if a stop's cancel stays pending past the in-sweep settle (~1s) and a cycle runs after it lands, the reconciler exits it (one exit, labelled UNPROTECTED); a position booked in the same cycle whose stop AND emergency exit both die could read held 0 from the cycle's positions snapshot and halt (fail closed).
-GATES: Full gate 28 Oct 2026, one pass: ruff check/format and mypy clean (STATIC EXIT CODE 0); 2,798 passed, 0 failed, 0 skipped (PYTEST EXIT CODE 0, written by the run itself); coverage 93% flat (squareoff 94%, service 96%, reconciliation 96%, positions 97%, trading models 98%); bandit exit 0; pip-audit exit 0 (7 accepted IDs), re-run before push; security suite 460 passed; doctor: only Datastores FAIL (dev machine). Two earlier runs were NOT green and are recorded: 14 failures reported through a pipe as exit 0 (QA-E15-37), and a mypy failure after the _is_the_exit refactor (fixed with TypeGuard).
+GATES: Full gate 28 Oct 2026, one pass: ruff check/format and mypy clean (STATIC EXIT CODE 0); 2,798 passed, 0 failed, 0 skipped (PYTEST EXIT CODE 0, written by the run itself); coverage 93% flat; bandit exit 0; pip-audit exit 0 (7 accepted IDs), re-run before push; gitleaks clean on the pushed range; security suite 460 passed; doctor: only Datastores FAIL (dev machine). Two earlier runs were NOT green and are recorded: 14 failures reported through a pipe as exit 0 (QA-E15-37), and a mypy failure after the _is_the_exit refactor (fixed with TypeGuard). CI: DEV Run 119 green (4c1ab92); promoted DEV 4c1ab92 -&gt; QA a9c971b via promote.py (exit 0; CI check passed, no divergence, stripped paths verified absent); QA Run 120 green.
 MUTATION: 30 named mutations over squareoff.py, the reconciler guard, positions.py, service.py and the Position validator: 30 killed, sources byte-identical (first run 26/29 + 2 never ran: QA-E15-38).
-SIT: Pending - SIT-21 (updated: every position now leaves at its deadline, closed TIME) and SIT-22 (a day with three positions and two deadlines, a restart after the deadline, a kill switch mid-session, yesterday's stale row) pass on DEV; to run on the QA tree.</t>
+SIT: SIT on the QA tree (worktree at origin/QA a9c971b, algotrader imported from the worktree), whole suite because the change spans components: 2,798 passed, 0 failed, 0 skipped, PYTEST EXIT CODE 0. SIT-22 walks the real stack (Postgres, Redis, Kite payloads): three positions across two deadlines each exit IN their deadline's minute, never with a stop and an exit both working, all closed TIME, flat at the close; a restart at 15:17 after a 15:15 deadline squares off at once, once, for what was held, closed TIME; a kill switch at 14:00 leaves the time exits untouched; yesterday's OPEN row halts the morning (POSITION_NOT_HELD) and nothing is sold all day. SIT-21 updated: every position now leaves at its deadline. No SIT defects.</t>
         </is>
       </c>
       <c r="W132" s="49" t="n"/>

</xml_diff>

<commit_message>
Record E15-S14's QA run
E15-S14 -> QA-Success: QA 29c06e7 (from DEV 251c5ac), DEV Run 122 and QA
Run 123 green, SIT on the QA tree 2,879 passed / 0 skipped, mutation 28/28.
Acceptance criteria rewritten as falsifiable; task 2's order-bucket wording
corrected with the reason. QA-E15-39..41, AUDIT-033 (autobahn
CVE-2026-116579, fixed) and AUDIT-034 (STRIDE). Concerns written onto
E13-S01 (publish before you emit), E15-S10 (the paper broker answers
margin_required), E23-S03 (how to compose LiveSessionFacts), E03-S01 (daily
bars must end on the previous session) and E20-S05 (health is the last
NoProducerYet input). B8 carries a 29 Oct observation: NSE refused this
host's home page while its archive and ban list answered.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documents/BACKLOG_Tracker.xlsx
+++ b/Documents/BACKLOG_Tracker.xlsx
@@ -7172,7 +7172,8 @@
       <c r="W32" s="49" t="n"/>
       <c r="X32" s="75" t="inlineStr">
         <is>
-          <t>NSE replaced the legacy bhavcopy with the UDiFF format and moved the URL. A fetcher written against the old path will 404, or worse fetch a stale mirror. Pin the exact source and assert on the header row, not just on HTTP 200. Also: bhavcopy is UNADJUSTED, so this must land before E03-S02 computes factors, never after.</t>
+          <t>NSE replaced the legacy bhavcopy with the UDiFF format and moved the URL. A fetcher written against the old path will 404, or worse fetch a stale mirror. Pin the exact source and assert on the header row, not just on HTTP 200. Also: bhavcopy is UNADJUSTED, so this must land before E03-S02 computes factors, never after.
+FROM E15-S14 (29 Oct 2026): correlations are computed from DAILY closes in ohlcv (timeframe 1d) and need every candidate's and held name's series to END ON THE PREVIOUS SESSION; a series that stops earlier makes its correlation unknown, and the guard then refuses any second position.</t>
         </is>
       </c>
     </row>
@@ -13849,7 +13850,8 @@
       <c r="W112" s="49" t="n"/>
       <c r="X112" s="75" t="inlineStr">
         <is>
-          <t>SEQUENCING BUG: this story is Phase 4 but depends on E12-S01 (strategy registry), which is Phase 5. Phase 4 cannot complete as currently sequenced. Either pull E12-S01 forward into Phase 4 or move this story into Phase 5.</t>
+          <t>SEQUENCING BUG: this story is Phase 4 but depends on E12-S01 (strategy registry), which is Phase 5. Phase 4 cannot complete as currently sequenced. Either pull E12-S01 forward into Phase 4 or move this story into Phase 5.
+FROM E15-S14 (29 Oct 2026): the execution service sizes every signal from the ATR this loop PUBLISHES. After folding each sealed bar into a symbol's IndicatorSet, call indicators.publish.publish_indicator_state BEFORE emitting any signal evaluated on that bar. Execution refuses a state older than one bar + 30s, not ready (warming or a feed gap), or on another timeframe than the signal's strategy declares - a signal that overtakes its own bar's state is refused.</t>
         </is>
       </c>
     </row>
@@ -16185,7 +16187,8 @@
       <c r="X136" s="75" t="inlineStr">
         <is>
           <t>'Switching paper-&gt;live changes exactly one dependency injection' is a strong claim and deserves a STRUCTURAL test, the way the ReadOnlyGuard test works. Otherwise one stray `if mode == PAPER` in the risk path makes every paper result unrepresentative of live.
-FROM E15-S13 (28 Oct 2026): the execution service sends in PAPER and LIVE modes to WHATEVER placer it is given - it cannot tell a paper placer from Kite. This story's placer is what makes PAPER safe: the entrypoint must hand the gateway the paper placer in PAPER mode, and nothing else may. ALERT_ONLY and APPROVAL are refused by the service itself (AUDIT-027).</t>
+FROM E15-S13 (28 Oct 2026): the execution service sends in PAPER and LIVE modes to WHATEVER placer it is given - it cannot tell a paper placer from Kite. This story's placer is what makes PAPER safe: the entrypoint must hand the gateway the paper placer in PAPER mode, and nothing else may. ALERT_ONLY and APPROVAL are refused by the service itself (AUDIT-027).
+FROM E15-S14 (29 Oct 2026): the paper broker must answer KiteTradingAdapter.margin_required(symbol, side=..., quantity=1) -&gt; Decimal - LiveSessionFacts' margin producer calls it in PAPER mode exactly as in LIVE. Zero or an error refuses the signal.</t>
         </is>
       </c>
     </row>
@@ -18814,7 +18817,8 @@
       <c r="W171" s="49" t="n"/>
       <c r="X171" t="inlineStr">
         <is>
-          <t>FROM E15-S13 (28 Oct 2026): the execution service asks SessionFacts.unhealthy_services(now=...) for the health roll-up; until this story provides it, NoProducerYet answers None and the engine rejects EVERY signal (HEALTH via RISK_ENGINE_FAULT). Implement it as a SessionFacts method returning a tuple of unhealthy service names - empty only when every service was checked.</t>
+          <t>FROM E15-S13 (28 Oct 2026): the execution service asks SessionFacts.unhealthy_services(now=...) for the health roll-up; until this story provides it, NoProducerYet answers None and the engine rejects EVERY signal (HEALTH via RISK_ENGINE_FAULT). Implement it as a SessionFacts method returning a tuple of unhealthy service names - empty only when every service was checked.
+FROM E15-S14 (29 Oct 2026): health is now the only live input without a producer. LiveSessionFacts takes it as `health` - an object with unhealthy_services(now=...) -&gt; tuple[str, ...] | None.</t>
         </is>
       </c>
     </row>
@@ -20304,7 +20308,8 @@
       <c r="X191" s="75" t="inlineStr">
         <is>
           <t>'Verify core has no internet access, by attempt' is the right test. Note the tension with E02-S01's auth callback and E17-S01's dashboard access — both want inbound reachability. Resolve the network design ONCE here rather than three times in three stories, or the answers will disagree.
-FROM E15-S13 (28 Oct 2026): docker-compose runs `python -m algotrader.execution`, and no service has a __main__ yet. The execution entrypoint composes ExecutionService (execution/service.py) with: the Kite trading adapter (or E15-S10's paper placer in PAPER mode - AUDIT-027), a session per operation for the repositories, RepositoryContextStore, HaltController, AuditWriter.write as the audit sink, and RedisSignalSource; then `await service.run(source, stop)`. QA-VER-01 constraint 4 lands here too: reconciliation reads must not share the data token bucket with backfill.</t>
+FROM E15-S13 (28 Oct 2026): docker-compose runs `python -m algotrader.execution`, and no service has a __main__ yet. The execution entrypoint composes ExecutionService (execution/service.py) with: the Kite trading adapter (or E15-S10's paper placer in PAPER mode - AUDIT-027), a session per operation for the repositories, RepositoryContextStore, HaltController, AuditWriter.write as the audit sink, and RedisSignalSource; then `await service.run(source, stop)`. QA-VER-01 constraint 4 lands here too: reconciliation reads must not share the data token bucket with backfill.
+FROM E15-S14 (29 Oct 2026): compose the service's facts as LiveSessionFacts(health=NoProducerYet() until E20-S05, atr=PublishedATR(redis, timeframes=strategy_timeframes(&lt;the strategy documents the strategy side loads&gt;)), margin=BrokerMarginPerShare(&lt;the trading adapter, or the paper one&gt;), correlations=DailyCloseCorrelations(BarRepository(...), calendar=...)).</t>
         </is>
       </c>
     </row>
@@ -21548,7 +21553,7 @@
       </c>
       <c r="E206" s="40" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>QA-Success</t>
         </is>
       </c>
       <c r="F206" s="41" t="inlineStr">
@@ -21601,14 +21606,25 @@
       </c>
       <c r="U206" s="48" t="inlineStr">
         <is>
-          <t>AC1 (RED) With the producers wired, an approvable signal is approved and sized from the live ATR and margin.
-AC2 (RED) A stale ATR, an unanswered margin call, or an uncomputable correlation each still rejects, naming the input.
-AC3 (RED) A held symbol whose correlation is unknown still refuses a second position.</t>
+          <t>AC1 (RED) With the producers wired - ATR from the state the real IndicatorSet publishes to Redis, margin from the Kite adapter's /margins/orders answer, correlations from daily closes in Postgres - an approvable signal is SUBMITTED, and its quantity is the sizer's from that ATR and margin (the risk budget over 1.5 x ATR; and the margin clamp when the broker's per-share margin is dear).
+AC2 (RED) Each of these rejects, places nothing, and the rejection detail names the input: no published state; a state more than one bar + 30s old; a signal from a strategy the service was not given; a margin call that fails; a zero margin.
+AC3 (RED) With a position held, a candidate whose daily history is missing, or does not end on the previous session, is refused (RISK_ENGINE_FAULT, naming the held symbol); the control - both histories current and uncorrelated - takes the second position.</t>
         </is>
       </c>
       <c r="V206" s="48" t="inlineStr">
         <is>
-          <t>RAISED 28 Oct 2026 by E15-S13. The service, the context builder and NoProducerYet exist; these three inputs are the reason production rejects every signal today (with E20-S05's health roll-up).</t>
+          <t>RAISED 28 Oct 2026 by E15-S13. The service, the context builder and NoProducerYet exist; these three inputs are the reason production rejects every signal today (with E20-S05's health roll-up).
+BUSINESS ANALYSIS, 29 Oct 2026 (/sdlc, E15-S14).
+DoR: R1 ok (P0, 2d, Safety-critical). R2 ok - E15-S13 QA-Success. R3 no blocker covers it (B8 blocks the daily-bar SOURCE, E03-S01, not this story). R4 LLA 4.1/4.3/5.7/8.3, session_context, sizer, correlation, the Kite adapter and the indicator engine read this session.
+VALUE: the inputs every approval is sized from. What breaks if wrong: a position sized from a stale or another strategy's ATR (every size wrong by the same factor, all day); a margin guessed low; two names that are one bet read as unrelated; margin lookups starving an exit order.
+TASK CORRECTIONS, recorded: (1) Task 1's ATR cannot be computed from Postgres - live bars reach it only after the session (LLA 4.1) - so the strategy side PUBLISHES its state (IndicatorSet.published -&gt; indicators/publish.py -&gt; state:indicator, an IndicatorSnapshot with as_of and ready) and execution reads it. (2) Task 2 said 'behind the order-rate limiter'; that would let a burst of margin lookups refuse an exit order. It is a read and takes a DATA token (KiteTradingAdapter.margin_required, asserted by a token-counting test).
+DECISIONS: ATR on the signal's own strategy's timeframe (strategy_timeframes from the strategy documents; an unknown strategy has no ATR); refused if absent, not ready, describing another key, dated &gt;5s ahead, or older than one bar + 30s. Margin: one share, NSE/MIS/MARKET, the signal's side, 5s bound (it runs under the lock the square-off timer takes), &lt;=0 is unknown. Correlations: daily closes, today's bar excluded, each pair ALIGNED ON COMMON DATES (correlations_against pairs by position - QA-E15-41), unknown for a series not ending on the previous session. SessionFacts.atr gains strategy_id and margin_per_share gains direction. Health stays NoProducerYet (E20-S05); LiveSessionFacts composes the four.
+OUT OF SCOPE, recorded: the health roll-up (E20-S05); calling the publisher from the strategy loop (E13-S01, concern written); the paper broker's margin (E15-S10, concern written); daily-bar ingestion (E03-S01, concern written); composing it at the entrypoint (E23-S03, concern written).
+RESIDUALS, recorded: margin is asked for every signal that reaches the context build, including ones a check then rejects (one read per signal); a 1h strategy's last bar of the day reports an as_of after 15:30 (no entry is possible then); the sizing ATR is atr_14 on the strategy's timeframe - a strategy wanting another needs the mapping from its stop primitive; the 30s grace is a judgement. In production every input is still unknown until E13-S01 publishes and E03 fills daily bars, and health until E20-S05.
+FOUND MID-STORY: autobahn CVE-2026-116579 (published 28 Oct 21:10 UTC) turned the dependency audit red; FIXED by moving every install site to 26.10.2, in its own commit (AUDIT-033).
+GATES: Full gate 29 Oct 2026, one pass after the venv repair (the first run failed to COLLECT: the autobahn replacement had been interrupted, pytest exit 2 - not a code failure, recorded in b96b167): 2,879 passed, 0 failed, 0 skipped, PYTEST EXIT 0, coverage 93% (flat; live_inputs 94%, publish 100%, session_context 93%); ruff check/format and mypy clean over the whole tree; bandit 0; pip-audit 0 with the 7 accepted IDs, re-run before push; security suite 461 passed; gitleaks clean on the 2 pushed commits; ops/Dockerfile image built and imports kiteconnect under autobahn 26.10.2; doctor: Configuration/Broker SDK/Market calendar/Strategies OK (Datastores FAIL and Secrets/SEBI/Network WARN are the dev machine). CI: DEV Run 122 green on 251c5ac (with b96b167 autobahn); promoted DEV 251c5ac -&gt; QA 29c06e7 via promote.py (CI check passed, no divergence, Documents/scripts/tracker/.claude stripped and verified absent); QA Run 123 green on 29c06e7.
+MUTATION: 28 named mutations across live_inputs, the Kite margin read, IndicatorSet.published/restore, the publisher and the context builder: 28 killed, sources byte-identical.
+SIT: SIT on the QA tree (detached worktree at origin/QA 29c06e7, algotrader imported from the worktree), whole suite because the change spans broker, indicators and execution: 2,879 passed, 0 failed, 0 skipped, PYTEST EXIT 0. SIT-23 (tests/sit/test_e15_execution_session.py) walks a day with the live producers wired - the strategy side publishing state each 5m bar, a TCS feed gap 11:00-12:00 then a re-warm, the margin desk down 13:00-13:10, HDFCBANK with no daily history - and asserts every signal ends one audited way: INFY, TCS (after the re-warm) and WIPRO (after the outage) submitted and sized from the published ATR; HDFCBANK refused naming the held INFY (correlation unknown); TCS during the gap refused naming its ATR; WIPRO during the outage refused naming its per-share margin; every entry protected by one stop, squared off once at its deadline and closed TIME; no halt. No SIT defects.</t>
         </is>
       </c>
       <c r="W206" s="49" t="n"/>
@@ -21712,6 +21728,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="59">
       <c r="A4" s="37" t="inlineStr">
         <is>
@@ -22140,7 +22157,8 @@
 It is a fetch-RELIABILITY problem, not a wall. The data is public; the difficulty is that the site is hostile to automation and changes shape without notice. Kite's instrument dump does NOT help - it carries token, symbol, tick size, lot size and segment, with no series, ASM, GSM, T2T or ban field (verified against the API docs).
 MITIGATIONS: jugaad-data (actively maintained, with caching specifically to avoid being blocked); nsefin for corporate actions, which is also E03-S02's missing feed; BSE as a fallback since ~90% of NSE equities are dual-listed; Zerodha's consolidated scrip sheet as a cross-check only (no SLA). The India-hosted VPS already required by constraint C1 sidesteps the geo-restriction.
 WHY IT IS SURVIVABLE: the fetch runs at 05:30, hours before the open, so a failure has a long runway for a retry, a fallback source or a manual override. E04-S01's acceptance criterion already says a fetch failure blocks the trading day rather than proceeding blind - the right posture: a bad fetch costs a trading day, not money.
-ACTION: spend an hour proving NSE reachability from the target environment before writing fetchers. That assumption sits under 8 stories and roughly 10 days of work.</t>
+ACTION: spend an hour proving NSE reachability from the target environment before writing fetchers. That assumption sits under 8 stories and roughly 10 days of work.
+OBSERVED 29 Oct 2026 (E15-S14 orientation): scripts/check_data_reachability.py from the development host (egress 14.96.14.58, an APNIC address) - NSE home 403 and the NSE ASM list an HTML interstitial, while the NSE bhavcopy archive, the NSE F&amp;O ban list, BSE and the Kite instruments dump all answered. If that host is in India, 'NSE blocks only overseas access' is incomplete and the India VPS may not resolve B8 by itself. Not concluded here; re-run on the VPS as planned.</t>
         </is>
       </c>
     </row>
@@ -22381,7 +22399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J160"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="59" min="1" max="1"/>
@@ -28324,6 +28342,117 @@
       <c r="G160" s="76" t="inlineStr">
         <is>
           <t>30 named mutations, 30 killed; sources byte-identical. tests/unit/test_squareoff.py::...test_a_stop_cancelled_part_filled_is_not_the_exit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="76" t="inlineStr">
+        <is>
+          <t>QA-E15-39</t>
+        </is>
+      </c>
+      <c r="B161" s="76" t="inlineStr">
+        <is>
+          <t>E15-S14</t>
+        </is>
+      </c>
+      <c r="C161" s="76" t="inlineStr">
+        <is>
+          <t>The first ATR design read a day-old number all session</t>
+        </is>
+      </c>
+      <c r="D161" s="76" t="inlineStr">
+        <is>
+          <t>FAIL -&gt; Fixed (design review)</t>
+        </is>
+      </c>
+      <c r="E161" s="76" t="inlineStr">
+        <is>
+          <t>The first design computed the ATR in execution from the bars in Postgres - self-contained and testable today. LLA 4.1 puts live bars in Redis streams during the session and flushes them to Postgres afterwards, so that ATR would be yesterday's for the whole session and every signal would be refused (or, with intraday backfill, sized off a stale range).</t>
+        </is>
+      </c>
+      <c r="F161" s="76" t="inlineStr">
+        <is>
+          <t>The strategy side publishes its own state (IndicatorSet.published, indicators/publish.py) to state:indicator with as_of and ready; execution reads the one for the signal's strategy and refuses anything older than one bar + 30s.</t>
+        </is>
+      </c>
+      <c r="G161" s="76" t="inlineStr">
+        <is>
+          <t>tests/unit/test_live_inputs.py::TestReadAtr, ::TestPublishedAtr::test_what_the_writer_publishes_the_reader_reads; integration TestS14Ac2...::test_a_stale_atr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="76" t="inlineStr">
+        <is>
+          <t>QA-E15-40</t>
+        </is>
+      </c>
+      <c r="B162" s="76" t="inlineStr">
+        <is>
+          <t>E15-S14</t>
+        </is>
+      </c>
+      <c r="C162" s="76" t="inlineStr">
+        <is>
+          <t>The story's task put margin lookups on the order-rate limiter</t>
+        </is>
+      </c>
+      <c r="D162" s="76" t="inlineStr">
+        <is>
+          <t>FAIL -&gt; Corrected (story)</t>
+        </is>
+      </c>
+      <c r="E162" s="76" t="inlineStr">
+        <is>
+          <t>Task 2 read 'Kite order_margins ... behind the order-rate limiter'. The order bucket is 3/s with a burst of 3 and exists so that nothing can starve an order; a margin lookup per signal there could refuse a stop or a time exit in the same second.</t>
+        </is>
+      </c>
+      <c r="F162" s="76" t="inlineStr">
+        <is>
+          <t>margin_required goes through the adapter's read path and takes a DATA token. The task is corrected on the story with the reason.</t>
+        </is>
+      </c>
+      <c r="G162" s="76" t="inlineStr">
+        <is>
+          <t>tests/unit/test_live_inputs.py::TestMarginRequired::test_it_takes_a_data_token_never_an_order_token; mutation 'margin on the order bucket' killed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="76" t="inlineStr">
+        <is>
+          <t>QA-E15-41</t>
+        </is>
+      </c>
+      <c r="B163" s="76" t="inlineStr">
+        <is>
+          <t>E15-S14</t>
+        </is>
+      </c>
+      <c r="C163" s="76" t="inlineStr">
+        <is>
+          <t>correlations_against pairs returns by position, not by date</t>
+        </is>
+      </c>
+      <c r="D163" s="76" t="inlineStr">
+        <is>
+          <t>FAIL -&gt; Fixed (producer)</t>
+        </is>
+      </c>
+      <c r="E163" s="76" t="inlineStr">
+        <is>
+          <t>correlations_against (E14-S04) pairs the tail of each series by POSITION, which is right only when both cover the same sessions. A name that did not trade for three sessions mid-window paired every older return with the wrong day's: a pair at 0.98 read below 0.7, i.e. one bet read as two.</t>
+        </is>
+      </c>
+      <c r="F163" s="76" t="inlineStr">
+        <is>
+          <t>The producer aligns each pair on the dates both traded before calling it (daily_correlations). correlations_against is unchanged; its callers are now the producer and tests.</t>
+        </is>
+      </c>
+      <c r="G163" s="76" t="inlineStr">
+        <is>
+          <t>tests/unit/test_live_inputs.py::TestDailyCorrelations::test_pairs_are_aligned_on_common_dates (asserts the by-position reading is &lt; 0.7 and the aligned one &gt; 0.9); mutation 'paired by position' killed.</t>
         </is>
       </c>
     </row>
@@ -28344,7 +28473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="59" min="1" max="1"/>
@@ -31975,6 +32104,90 @@
       <c r="H87" s="76" t="inlineStr">
         <is>
           <t>tests/unit/test_squareoff.py::TestItsMemoryIsBounded; mutation 'memory never pruned' killed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="76" t="inlineStr">
+        <is>
+          <t>AUDIT-033</t>
+        </is>
+      </c>
+      <c r="B88" s="76" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C88" s="76" t="inlineStr">
+        <is>
+          <t>dependency autobahn 26.7.1 - CVE-2026-116579 / GHSA-pjh6-c8mg-3x7m</t>
+        </is>
+      </c>
+      <c r="D88" s="76" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="E88" s="76" t="inlineStr">
+        <is>
+          <t>Published 28 Oct 2026 21:10 UTC; the dependency audit went red mid-story. permessage-brotli inflates a whole frame before maxMessagePayloadSize is checked, so one 421-byte frame costs an autobahn SERVER ~545 MiB.</t>
+        </is>
+      </c>
+      <c r="F88" s="76" t="inlineStr">
+        <is>
+          <t>Unreachable here: this system runs no autobahn server, enables no WebSocket compression extension, and never constructs a KiteTicker (autobahn is present only because kiteconnect imports its ticker module).</t>
+        </is>
+      </c>
+      <c r="G88" s="76" t="inlineStr">
+        <is>
+          <t>Fixed anyway, because a fix exists: every install site (ci.yml x3, ops/Dockerfile, Makefile, docs) moves to 26.10.2; requirements (cryptography&gt;=50, cbor2&gt;=6.1, txaio&gt;=25.12.2) already met by constraints.txt. kiteconnect 5.2.1 verified under it (imports, login URL, market_protection/algo_id, ticker import), locally and inside the built runtime image.</t>
+        </is>
+      </c>
+      <c r="H88" s="76" t="inlineStr">
+        <is>
+          <t>tests/security/test_dependency_hygiene.py::TestAutobahnIsNotTheVulnerableVersion::test_the_installed_autobahn_carries_the_brotli_fix (BROTLI_FIX_AUTOBAHN = 26.10.1); pip-audit clean with the same 7 accepted IDs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="76" t="inlineStr">
+        <is>
+          <t>AUDIT-034</t>
+        </is>
+      </c>
+      <c r="B89" s="76" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C89" s="76" t="inlineStr">
+        <is>
+          <t>execution/live_inputs.py, indicators/publish.py, KiteTradingAdapter.margin_required - STRIDE</t>
+        </is>
+      </c>
+      <c r="D89" s="76" t="inlineStr">
+        <is>
+          <t>Assessed</t>
+        </is>
+      </c>
+      <c r="E89" s="76" t="inlineStr">
+        <is>
+          <t>S: the published state must match its key (symbol, timeframe), be ready, not be from the future, and be at most one bar + 30s old. A tampered ATR cannot breach the per-trade risk bound: quantity x stop &lt;= budget holds for ANY ATR, a vanishing ATR sizes a zero-width stop (refused) and a huge one puts the stop past the entry (refused). T: the state is validated by IndicatorSnapshot (NaN/inf refused, probed); -0 refused by the reader; the margin total must be one finite row for the symbol asked. R: every refusal names the input in decision_log; the producer logs why. I: logs go through one_safe_line; the audit detail carries the RiskContextError message, never broker text. D: per signal one Redis GET, one broker read (5s bound, data bucket) and one DB query; the timer waits at most one signal for the lock. E: strategy_id selects a timeframe by dict lookup (unknown -&gt; None); the symbol reaches a Redis key only through keys._safe.</t>
+        </is>
+      </c>
+      <c r="F89" s="76" t="inlineStr">
+        <is>
+          <t>Residuals recorded on E15-S14.</t>
+        </is>
+      </c>
+      <c r="G89" s="76" t="inlineStr">
+        <is>
+          <t>None required beyond the story.</t>
+        </is>
+      </c>
+      <c r="H89" s="76" t="inlineStr">
+        <is>
+          <t>tests/unit/test_live_inputs.py (67), integration TestS14* (10), SIT-23; mutation 28/28.</t>
         </is>
       </c>
     </row>

</xml_diff>